<commit_message>
Match 1 & 2
</commit_message>
<xml_diff>
--- a/matches.xlsx
+++ b/matches.xlsx
@@ -8,20 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vs\world_cup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A49FF4-59ED-4FFE-BF8A-A26F3EDDABC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241C0460-3E73-48BC-910D-4614BEBB773B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5129E331-5CE9-4084-9F59-05652B25F4C8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5129E331-5CE9-4084-9F59-05652B25F4C8}"/>
   </bookViews>
   <sheets>
     <sheet name="WC_2026" sheetId="1" r:id="rId1"/>
     <sheet name="Historic_Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="126">
   <si>
     <t>Date</t>
   </si>
@@ -1240,11 +1251,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0676E7-9C9C-4876-9697-3A2602566485}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -1292,9 +1303,75 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46185</v>
+      </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2">
+        <v>1881</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G2">
+        <v>1511</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
       <c r="K2">
         <f>IF(E2&gt;H2, 2, IF(E2=H2, 1, 0))</f>
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46185</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3">
+        <v>1758</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3">
+        <v>1740</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <f>IF(E3&gt;H3, 2, IF(E3=H3, 1, 0))</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>